<commit_message>
Add wish input feature with dropdown
希望休入力機能の改善（プルダウン、曜日表示、None削除、罫線追加）
</commit_message>
<xml_diff>
--- a/Shift_Input.xlsx
+++ b/Shift_Input.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sim95\Desktop\shift_project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ffeeb9b519dc77a8/shift_project/shift-optimizer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43A4AF22-E5D3-4CA7-8324-C4DD0CACD583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{43A4AF22-E5D3-4CA7-8324-C4DD0CACD583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BDDBA1A-85BE-4D8C-8BD0-594D9218BF4A}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="450" windowWidth="15780" windowHeight="14535" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1905" yWindow="450" windowWidth="15780" windowHeight="14535" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="設定" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="32">
   <si>
     <t>年</t>
   </si>
@@ -1795,7 +1795,9 @@
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
+      <c r="H5" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6">
@@ -1943,7 +1945,9 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
+      <c r="H14" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="6">

</xml_diff>